<commit_message>
NW final v2: empty-state RULE adopted (full layout w/ zeros, ONE app-wide retirement sample) — State C redrawn; UX v1.2 rule row + changelog row
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-UX-design-v1.2-2026-08-04.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-UX-design-v1.2-2026-08-04.xlsx
@@ -953,7 +953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1136,6 +1136,23 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>One scannable ledger grammar everywhere; numbers always share a right edge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EMPTY-STATE RULE (founder 2026-08-04)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>When data is missing, keep the FULL layout: real structure with $0 values (Own $0 − Owe $0 = $0), every band/section in place, and the door to add data. Concepts with a sample first-view use ONE app-wide sample — the Home retirement sample ("Sample: 84% odds of lasting to age 90 — a sample, not your number") is THE retirement first-view everywhere. Never reinvent an empty state per screen.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A stripped empty screen teaches nothing; the full layout with zeros shows what the screen becomes and how to move forward. One sample per concept keeps the app consistent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FIFTH INGREDIENT CHECK: history_from recorded at ingest (depth only deepens) + historyCoverage() one-sentence labeling wired to the 12-month investment-income figure; 10 pins; 1416 green; UX + changelog rows
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-UX-design-v1.2-2026-08-04.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-UX-design-v1.2-2026-08-04.xlsx
@@ -1167,7 +1167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1371,6 +1371,23 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Direct labels are the colorblind relief the validator requires; the classification rule protects change/ROI accuracy (founder decision, supersedes money-market=cash and the 12-month CD split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>History-depth labeling (founder 2026-08-04)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Any figure spanning a year or more names the coverage its sources actually shared, one sentence per source, directly under the figure. Silent when coverage is complete. Window figures (walks, returns) never include rows dated before the window; income figures count any dated receipt the source vouches for, including pre-join back-fill.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Brokers back-fill different depths; an unlabeled "past year" total silently understates.</t>
         </is>
       </c>
     </row>

</xml_diff>